<commit_message>
Agregar campos de isocronas de salud a plataforma enie
</commit_message>
<xml_diff>
--- a/riobamba-censo-data/shp/plataforma_enie.xlsx
+++ b/riobamba-censo-data/shp/plataforma_enie.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Datos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Datos'!$A$1:$AG$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Datos'!$A$1:$AI$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG198"/>
+  <dimension ref="A1:AI198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -526,6 +526,8 @@
     <col width="24" customWidth="1" min="31" max="31"/>
     <col width="24" customWidth="1" min="32" max="32"/>
     <col width="24" customWidth="1" min="33" max="33"/>
+    <col width="24" customWidth="1" min="34" max="34"/>
+    <col width="24" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -694,6 +696,16 @@
           <t>iso_nom_22</t>
         </is>
       </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>sal_nom_1</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>sal_nom_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -835,6 +847,12 @@
       </c>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -972,6 +990,8 @@
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1109,6 +1129,12 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1206,6 +1232,8 @@
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1303,6 +1331,8 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1388,6 +1418,8 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1481,6 +1513,8 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1618,6 +1652,8 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1747,6 +1783,8 @@
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1880,6 +1918,8 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2009,6 +2049,8 @@
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2146,6 +2188,8 @@
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2295,6 +2339,8 @@
           <t>iso_087_parada_400m_PARADA_BUS_087_Parada_087_-_Lineas_16</t>
         </is>
       </c>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2440,6 +2486,8 @@
         </is>
       </c>
       <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2577,6 +2625,8 @@
       <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr"/>
       <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2726,6 +2776,8 @@
           <t>iso_046_parada_400m_PARADA_BUS_046_Parada_046_-_Lineas_07_10</t>
         </is>
       </c>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2807,6 +2859,8 @@
       <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr"/>
       <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2880,6 +2934,8 @@
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr"/>
       <c r="AG19" t="inlineStr"/>
+      <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2965,6 +3021,8 @@
       <c r="AE20" t="inlineStr"/>
       <c r="AF20" t="inlineStr"/>
       <c r="AG20" t="inlineStr"/>
+      <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3042,6 +3100,8 @@
       <c r="AE21" t="inlineStr"/>
       <c r="AF21" t="inlineStr"/>
       <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3127,6 +3187,8 @@
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr"/>
       <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3264,6 +3326,8 @@
       <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr"/>
       <c r="AG23" t="inlineStr"/>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3397,6 +3461,8 @@
       <c r="AE24" t="inlineStr"/>
       <c r="AF24" t="inlineStr"/>
       <c r="AG24" t="inlineStr"/>
+      <c r="AH24" t="inlineStr"/>
+      <c r="AI24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3534,6 +3600,8 @@
       <c r="AE25" t="inlineStr"/>
       <c r="AF25" t="inlineStr"/>
       <c r="AG25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr"/>
+      <c r="AI25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3619,6 +3687,8 @@
       <c r="AE26" t="inlineStr"/>
       <c r="AF26" t="inlineStr"/>
       <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr"/>
+      <c r="AI26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3720,6 +3790,8 @@
       <c r="AE27" t="inlineStr"/>
       <c r="AF27" t="inlineStr"/>
       <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="inlineStr"/>
+      <c r="AI27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3821,6 +3893,8 @@
       <c r="AE28" t="inlineStr"/>
       <c r="AF28" t="inlineStr"/>
       <c r="AG28" t="inlineStr"/>
+      <c r="AH28" t="inlineStr"/>
+      <c r="AI28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3906,6 +3980,8 @@
       <c r="AE29" t="inlineStr"/>
       <c r="AF29" t="inlineStr"/>
       <c r="AG29" t="inlineStr"/>
+      <c r="AH29" t="inlineStr"/>
+      <c r="AI29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3987,6 +4063,8 @@
       <c r="AE30" t="inlineStr"/>
       <c r="AF30" t="inlineStr"/>
       <c r="AG30" t="inlineStr"/>
+      <c r="AH30" t="inlineStr"/>
+      <c r="AI30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4068,6 +4146,8 @@
       <c r="AE31" t="inlineStr"/>
       <c r="AF31" t="inlineStr"/>
       <c r="AG31" t="inlineStr"/>
+      <c r="AH31" t="inlineStr"/>
+      <c r="AI31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4149,6 +4229,8 @@
       <c r="AE32" t="inlineStr"/>
       <c r="AF32" t="inlineStr"/>
       <c r="AG32" t="inlineStr"/>
+      <c r="AH32" t="inlineStr"/>
+      <c r="AI32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4218,6 +4300,8 @@
       <c r="AE33" t="inlineStr"/>
       <c r="AF33" t="inlineStr"/>
       <c r="AG33" t="inlineStr"/>
+      <c r="AH33" t="inlineStr"/>
+      <c r="AI33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4303,6 +4387,8 @@
       <c r="AE34" t="inlineStr"/>
       <c r="AF34" t="inlineStr"/>
       <c r="AG34" t="inlineStr"/>
+      <c r="AH34" t="inlineStr"/>
+      <c r="AI34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4416,6 +4502,8 @@
       <c r="AE35" t="inlineStr"/>
       <c r="AF35" t="inlineStr"/>
       <c r="AG35" t="inlineStr"/>
+      <c r="AH35" t="inlineStr"/>
+      <c r="AI35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4505,6 +4593,8 @@
       <c r="AE36" t="inlineStr"/>
       <c r="AF36" t="inlineStr"/>
       <c r="AG36" t="inlineStr"/>
+      <c r="AH36" t="inlineStr"/>
+      <c r="AI36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4598,6 +4688,12 @@
       <c r="AE37" t="inlineStr"/>
       <c r="AF37" t="inlineStr"/>
       <c r="AG37" t="inlineStr"/>
+      <c r="AH37" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4687,6 +4783,12 @@
       <c r="AE38" t="inlineStr"/>
       <c r="AF38" t="inlineStr"/>
       <c r="AG38" t="inlineStr"/>
+      <c r="AH38" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4780,6 +4882,8 @@
       <c r="AE39" t="inlineStr"/>
       <c r="AF39" t="inlineStr"/>
       <c r="AG39" t="inlineStr"/>
+      <c r="AH39" t="inlineStr"/>
+      <c r="AI39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4853,6 +4957,8 @@
       <c r="AE40" t="inlineStr"/>
       <c r="AF40" t="inlineStr"/>
       <c r="AG40" t="inlineStr"/>
+      <c r="AH40" t="inlineStr"/>
+      <c r="AI40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4934,6 +5040,8 @@
       <c r="AE41" t="inlineStr"/>
       <c r="AF41" t="inlineStr"/>
       <c r="AG41" t="inlineStr"/>
+      <c r="AH41" t="inlineStr"/>
+      <c r="AI41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5015,6 +5123,8 @@
       <c r="AE42" t="inlineStr"/>
       <c r="AF42" t="inlineStr"/>
       <c r="AG42" t="inlineStr"/>
+      <c r="AH42" t="inlineStr"/>
+      <c r="AI42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5088,6 +5198,8 @@
       <c r="AE43" t="inlineStr"/>
       <c r="AF43" t="inlineStr"/>
       <c r="AG43" t="inlineStr"/>
+      <c r="AH43" t="inlineStr"/>
+      <c r="AI43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5165,6 +5277,8 @@
       <c r="AE44" t="inlineStr"/>
       <c r="AF44" t="inlineStr"/>
       <c r="AG44" t="inlineStr"/>
+      <c r="AH44" t="inlineStr"/>
+      <c r="AI44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5242,6 +5356,8 @@
       <c r="AE45" t="inlineStr"/>
       <c r="AF45" t="inlineStr"/>
       <c r="AG45" t="inlineStr"/>
+      <c r="AH45" t="inlineStr"/>
+      <c r="AI45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5311,6 +5427,8 @@
       <c r="AE46" t="inlineStr"/>
       <c r="AF46" t="inlineStr"/>
       <c r="AG46" t="inlineStr"/>
+      <c r="AH46" t="inlineStr"/>
+      <c r="AI46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5400,6 +5518,8 @@
       <c r="AE47" t="inlineStr"/>
       <c r="AF47" t="inlineStr"/>
       <c r="AG47" t="inlineStr"/>
+      <c r="AH47" t="inlineStr"/>
+      <c r="AI47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5485,6 +5605,8 @@
       <c r="AE48" t="inlineStr"/>
       <c r="AF48" t="inlineStr"/>
       <c r="AG48" t="inlineStr"/>
+      <c r="AH48" t="inlineStr"/>
+      <c r="AI48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5586,6 +5708,12 @@
       <c r="AE49" t="inlineStr"/>
       <c r="AF49" t="inlineStr"/>
       <c r="AG49" t="inlineStr"/>
+      <c r="AH49" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5695,6 +5823,12 @@
       <c r="AE50" t="inlineStr"/>
       <c r="AF50" t="inlineStr"/>
       <c r="AG50" t="inlineStr"/>
+      <c r="AH50" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5804,6 +5938,12 @@
       <c r="AE51" t="inlineStr"/>
       <c r="AF51" t="inlineStr"/>
       <c r="AG51" t="inlineStr"/>
+      <c r="AH51" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5909,6 +6049,12 @@
       <c r="AE52" t="inlineStr"/>
       <c r="AF52" t="inlineStr"/>
       <c r="AG52" t="inlineStr"/>
+      <c r="AH52" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6022,6 +6168,12 @@
       <c r="AE53" t="inlineStr"/>
       <c r="AF53" t="inlineStr"/>
       <c r="AG53" t="inlineStr"/>
+      <c r="AH53" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6151,6 +6303,12 @@
       <c r="AE54" t="inlineStr"/>
       <c r="AF54" t="inlineStr"/>
       <c r="AG54" t="inlineStr"/>
+      <c r="AH54" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6228,6 +6386,8 @@
       <c r="AE55" t="inlineStr"/>
       <c r="AF55" t="inlineStr"/>
       <c r="AG55" t="inlineStr"/>
+      <c r="AH55" t="inlineStr"/>
+      <c r="AI55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6313,6 +6473,8 @@
       <c r="AE56" t="inlineStr"/>
       <c r="AF56" t="inlineStr"/>
       <c r="AG56" t="inlineStr"/>
+      <c r="AH56" t="inlineStr"/>
+      <c r="AI56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6398,6 +6560,8 @@
       <c r="AE57" t="inlineStr"/>
       <c r="AF57" t="inlineStr"/>
       <c r="AG57" t="inlineStr"/>
+      <c r="AH57" t="inlineStr"/>
+      <c r="AI57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6483,6 +6647,8 @@
       <c r="AE58" t="inlineStr"/>
       <c r="AF58" t="inlineStr"/>
       <c r="AG58" t="inlineStr"/>
+      <c r="AH58" t="inlineStr"/>
+      <c r="AI58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6568,6 +6734,8 @@
       <c r="AE59" t="inlineStr"/>
       <c r="AF59" t="inlineStr"/>
       <c r="AG59" t="inlineStr"/>
+      <c r="AH59" t="inlineStr"/>
+      <c r="AI59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6649,6 +6817,8 @@
       <c r="AE60" t="inlineStr"/>
       <c r="AF60" t="inlineStr"/>
       <c r="AG60" t="inlineStr"/>
+      <c r="AH60" t="inlineStr"/>
+      <c r="AI60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6730,6 +6900,8 @@
       <c r="AE61" t="inlineStr"/>
       <c r="AF61" t="inlineStr"/>
       <c r="AG61" t="inlineStr"/>
+      <c r="AH61" t="inlineStr"/>
+      <c r="AI61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6811,6 +6983,8 @@
       <c r="AE62" t="inlineStr"/>
       <c r="AF62" t="inlineStr"/>
       <c r="AG62" t="inlineStr"/>
+      <c r="AH62" t="inlineStr"/>
+      <c r="AI62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6888,6 +7062,8 @@
       <c r="AE63" t="inlineStr"/>
       <c r="AF63" t="inlineStr"/>
       <c r="AG63" t="inlineStr"/>
+      <c r="AH63" t="inlineStr"/>
+      <c r="AI63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6969,6 +7145,8 @@
       <c r="AE64" t="inlineStr"/>
       <c r="AF64" t="inlineStr"/>
       <c r="AG64" t="inlineStr"/>
+      <c r="AH64" t="inlineStr"/>
+      <c r="AI64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7050,6 +7228,8 @@
       <c r="AE65" t="inlineStr"/>
       <c r="AF65" t="inlineStr"/>
       <c r="AG65" t="inlineStr"/>
+      <c r="AH65" t="inlineStr"/>
+      <c r="AI65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7131,6 +7311,8 @@
       <c r="AE66" t="inlineStr"/>
       <c r="AF66" t="inlineStr"/>
       <c r="AG66" t="inlineStr"/>
+      <c r="AH66" t="inlineStr"/>
+      <c r="AI66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7204,6 +7386,8 @@
       <c r="AE67" t="inlineStr"/>
       <c r="AF67" t="inlineStr"/>
       <c r="AG67" t="inlineStr"/>
+      <c r="AH67" t="inlineStr"/>
+      <c r="AI67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7281,6 +7465,8 @@
       <c r="AE68" t="inlineStr"/>
       <c r="AF68" t="inlineStr"/>
       <c r="AG68" t="inlineStr"/>
+      <c r="AH68" t="inlineStr"/>
+      <c r="AI68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7366,6 +7552,8 @@
       <c r="AE69" t="inlineStr"/>
       <c r="AF69" t="inlineStr"/>
       <c r="AG69" t="inlineStr"/>
+      <c r="AH69" t="inlineStr"/>
+      <c r="AI69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -7451,6 +7639,8 @@
       <c r="AE70" t="inlineStr"/>
       <c r="AF70" t="inlineStr"/>
       <c r="AG70" t="inlineStr"/>
+      <c r="AH70" t="inlineStr"/>
+      <c r="AI70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -7536,6 +7726,8 @@
       <c r="AE71" t="inlineStr"/>
       <c r="AF71" t="inlineStr"/>
       <c r="AG71" t="inlineStr"/>
+      <c r="AH71" t="inlineStr"/>
+      <c r="AI71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -7625,6 +7817,8 @@
       <c r="AE72" t="inlineStr"/>
       <c r="AF72" t="inlineStr"/>
       <c r="AG72" t="inlineStr"/>
+      <c r="AH72" t="inlineStr"/>
+      <c r="AI72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -7730,6 +7924,8 @@
       <c r="AE73" t="inlineStr"/>
       <c r="AF73" t="inlineStr"/>
       <c r="AG73" t="inlineStr"/>
+      <c r="AH73" t="inlineStr"/>
+      <c r="AI73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7823,6 +8019,8 @@
       <c r="AE74" t="inlineStr"/>
       <c r="AF74" t="inlineStr"/>
       <c r="AG74" t="inlineStr"/>
+      <c r="AH74" t="inlineStr"/>
+      <c r="AI74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7884,6 +8082,8 @@
       <c r="AE75" t="inlineStr"/>
       <c r="AF75" t="inlineStr"/>
       <c r="AG75" t="inlineStr"/>
+      <c r="AH75" t="inlineStr"/>
+      <c r="AI75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -7977,6 +8177,12 @@
       <c r="AE76" t="inlineStr"/>
       <c r="AF76" t="inlineStr"/>
       <c r="AG76" t="inlineStr"/>
+      <c r="AH76" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -8066,6 +8272,8 @@
       <c r="AE77" t="inlineStr"/>
       <c r="AF77" t="inlineStr"/>
       <c r="AG77" t="inlineStr"/>
+      <c r="AH77" t="inlineStr"/>
+      <c r="AI77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -8159,6 +8367,8 @@
       <c r="AE78" t="inlineStr"/>
       <c r="AF78" t="inlineStr"/>
       <c r="AG78" t="inlineStr"/>
+      <c r="AH78" t="inlineStr"/>
+      <c r="AI78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8248,6 +8458,8 @@
       <c r="AE79" t="inlineStr"/>
       <c r="AF79" t="inlineStr"/>
       <c r="AG79" t="inlineStr"/>
+      <c r="AH79" t="inlineStr"/>
+      <c r="AI79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -8341,6 +8553,8 @@
       <c r="AE80" t="inlineStr"/>
       <c r="AF80" t="inlineStr"/>
       <c r="AG80" t="inlineStr"/>
+      <c r="AH80" t="inlineStr"/>
+      <c r="AI80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -8418,6 +8632,12 @@
       <c r="AE81" t="inlineStr"/>
       <c r="AF81" t="inlineStr"/>
       <c r="AG81" t="inlineStr"/>
+      <c r="AH81" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -8495,6 +8715,8 @@
       <c r="AE82" t="inlineStr"/>
       <c r="AF82" t="inlineStr"/>
       <c r="AG82" t="inlineStr"/>
+      <c r="AH82" t="inlineStr"/>
+      <c r="AI82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -8576,6 +8798,8 @@
       <c r="AE83" t="inlineStr"/>
       <c r="AF83" t="inlineStr"/>
       <c r="AG83" t="inlineStr"/>
+      <c r="AH83" t="inlineStr"/>
+      <c r="AI83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -8649,6 +8873,8 @@
       <c r="AE84" t="inlineStr"/>
       <c r="AF84" t="inlineStr"/>
       <c r="AG84" t="inlineStr"/>
+      <c r="AH84" t="inlineStr"/>
+      <c r="AI84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -8726,6 +8952,8 @@
       <c r="AE85" t="inlineStr"/>
       <c r="AF85" t="inlineStr"/>
       <c r="AG85" t="inlineStr"/>
+      <c r="AH85" t="inlineStr"/>
+      <c r="AI85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -8803,6 +9031,8 @@
       <c r="AE86" t="inlineStr"/>
       <c r="AF86" t="inlineStr"/>
       <c r="AG86" t="inlineStr"/>
+      <c r="AH86" t="inlineStr"/>
+      <c r="AI86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -8876,6 +9106,8 @@
       <c r="AE87" t="inlineStr"/>
       <c r="AF87" t="inlineStr"/>
       <c r="AG87" t="inlineStr"/>
+      <c r="AH87" t="inlineStr"/>
+      <c r="AI87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -8937,6 +9169,8 @@
       <c r="AE88" t="inlineStr"/>
       <c r="AF88" t="inlineStr"/>
       <c r="AG88" t="inlineStr"/>
+      <c r="AH88" t="inlineStr"/>
+      <c r="AI88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -8998,6 +9232,8 @@
       <c r="AE89" t="inlineStr"/>
       <c r="AF89" t="inlineStr"/>
       <c r="AG89" t="inlineStr"/>
+      <c r="AH89" t="inlineStr"/>
+      <c r="AI89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -9083,6 +9319,16 @@
       <c r="AE90" t="inlineStr"/>
       <c r="AF90" t="inlineStr"/>
       <c r="AG90" t="inlineStr"/>
+      <c r="AH90" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI90" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -9164,6 +9410,16 @@
       <c r="AE91" t="inlineStr"/>
       <c r="AF91" t="inlineStr"/>
       <c r="AG91" t="inlineStr"/>
+      <c r="AH91" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI91" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -9245,6 +9501,16 @@
       <c r="AE92" t="inlineStr"/>
       <c r="AF92" t="inlineStr"/>
       <c r="AG92" t="inlineStr"/>
+      <c r="AH92" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI92" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -9322,6 +9588,16 @@
       <c r="AE93" t="inlineStr"/>
       <c r="AF93" t="inlineStr"/>
       <c r="AG93" t="inlineStr"/>
+      <c r="AH93" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI93" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -9403,6 +9679,16 @@
       <c r="AE94" t="inlineStr"/>
       <c r="AF94" t="inlineStr"/>
       <c r="AG94" t="inlineStr"/>
+      <c r="AH94" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI94" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -9484,6 +9770,12 @@
       <c r="AE95" t="inlineStr"/>
       <c r="AF95" t="inlineStr"/>
       <c r="AG95" t="inlineStr"/>
+      <c r="AH95" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -9565,6 +9857,12 @@
       <c r="AE96" t="inlineStr"/>
       <c r="AF96" t="inlineStr"/>
       <c r="AG96" t="inlineStr"/>
+      <c r="AH96" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -9642,6 +9940,12 @@
       <c r="AE97" t="inlineStr"/>
       <c r="AF97" t="inlineStr"/>
       <c r="AG97" t="inlineStr"/>
+      <c r="AH97" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -9723,6 +10027,8 @@
       <c r="AE98" t="inlineStr"/>
       <c r="AF98" t="inlineStr"/>
       <c r="AG98" t="inlineStr"/>
+      <c r="AH98" t="inlineStr"/>
+      <c r="AI98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -9812,6 +10118,8 @@
       <c r="AE99" t="inlineStr"/>
       <c r="AF99" t="inlineStr"/>
       <c r="AG99" t="inlineStr"/>
+      <c r="AH99" t="inlineStr"/>
+      <c r="AI99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -9917,6 +10225,12 @@
       <c r="AE100" t="inlineStr"/>
       <c r="AF100" t="inlineStr"/>
       <c r="AG100" t="inlineStr"/>
+      <c r="AH100" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -10010,6 +10324,12 @@
       <c r="AE101" t="inlineStr"/>
       <c r="AF101" t="inlineStr"/>
       <c r="AG101" t="inlineStr"/>
+      <c r="AH101" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -10095,6 +10415,12 @@
       <c r="AE102" t="inlineStr"/>
       <c r="AF102" t="inlineStr"/>
       <c r="AG102" t="inlineStr"/>
+      <c r="AH102" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -10196,6 +10522,12 @@
       <c r="AE103" t="inlineStr"/>
       <c r="AF103" t="inlineStr"/>
       <c r="AG103" t="inlineStr"/>
+      <c r="AH103" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -10301,6 +10633,12 @@
       <c r="AE104" t="inlineStr"/>
       <c r="AF104" t="inlineStr"/>
       <c r="AG104" t="inlineStr"/>
+      <c r="AH104" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -10398,6 +10736,12 @@
       <c r="AE105" t="inlineStr"/>
       <c r="AF105" t="inlineStr"/>
       <c r="AG105" t="inlineStr"/>
+      <c r="AH105" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -10491,6 +10835,8 @@
       <c r="AE106" t="inlineStr"/>
       <c r="AF106" t="inlineStr"/>
       <c r="AG106" t="inlineStr"/>
+      <c r="AH106" t="inlineStr"/>
+      <c r="AI106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -10552,6 +10898,8 @@
       <c r="AE107" t="inlineStr"/>
       <c r="AF107" t="inlineStr"/>
       <c r="AG107" t="inlineStr"/>
+      <c r="AH107" t="inlineStr"/>
+      <c r="AI107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -10645,6 +10993,8 @@
       <c r="AE108" t="inlineStr"/>
       <c r="AF108" t="inlineStr"/>
       <c r="AG108" t="inlineStr"/>
+      <c r="AH108" t="inlineStr"/>
+      <c r="AI108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -10730,6 +11080,8 @@
       <c r="AE109" t="inlineStr"/>
       <c r="AF109" t="inlineStr"/>
       <c r="AG109" t="inlineStr"/>
+      <c r="AH109" t="inlineStr"/>
+      <c r="AI109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -10823,6 +11175,8 @@
       <c r="AE110" t="inlineStr"/>
       <c r="AF110" t="inlineStr"/>
       <c r="AG110" t="inlineStr"/>
+      <c r="AH110" t="inlineStr"/>
+      <c r="AI110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -10888,6 +11242,8 @@
       <c r="AE111" t="inlineStr"/>
       <c r="AF111" t="inlineStr"/>
       <c r="AG111" t="inlineStr"/>
+      <c r="AH111" t="inlineStr"/>
+      <c r="AI111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -10949,6 +11305,8 @@
       <c r="AE112" t="inlineStr"/>
       <c r="AF112" t="inlineStr"/>
       <c r="AG112" t="inlineStr"/>
+      <c r="AH112" t="inlineStr"/>
+      <c r="AI112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -11010,6 +11368,8 @@
       <c r="AE113" t="inlineStr"/>
       <c r="AF113" t="inlineStr"/>
       <c r="AG113" t="inlineStr"/>
+      <c r="AH113" t="inlineStr"/>
+      <c r="AI113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -11095,6 +11455,8 @@
       <c r="AE114" t="inlineStr"/>
       <c r="AF114" t="inlineStr"/>
       <c r="AG114" t="inlineStr"/>
+      <c r="AH114" t="inlineStr"/>
+      <c r="AI114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -11180,6 +11542,8 @@
       <c r="AE115" t="inlineStr"/>
       <c r="AF115" t="inlineStr"/>
       <c r="AG115" t="inlineStr"/>
+      <c r="AH115" t="inlineStr"/>
+      <c r="AI115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -11265,6 +11629,8 @@
       <c r="AE116" t="inlineStr"/>
       <c r="AF116" t="inlineStr"/>
       <c r="AG116" t="inlineStr"/>
+      <c r="AH116" t="inlineStr"/>
+      <c r="AI116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -11350,6 +11716,8 @@
       <c r="AE117" t="inlineStr"/>
       <c r="AF117" t="inlineStr"/>
       <c r="AG117" t="inlineStr"/>
+      <c r="AH117" t="inlineStr"/>
+      <c r="AI117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -11427,6 +11795,8 @@
       <c r="AE118" t="inlineStr"/>
       <c r="AF118" t="inlineStr"/>
       <c r="AG118" t="inlineStr"/>
+      <c r="AH118" t="inlineStr"/>
+      <c r="AI118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -11540,6 +11910,12 @@
       <c r="AE119" t="inlineStr"/>
       <c r="AF119" t="inlineStr"/>
       <c r="AG119" t="inlineStr"/>
+      <c r="AH119" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -11641,6 +12017,12 @@
       <c r="AE120" t="inlineStr"/>
       <c r="AF120" t="inlineStr"/>
       <c r="AG120" t="inlineStr"/>
+      <c r="AH120" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -11750,6 +12132,12 @@
       <c r="AE121" t="inlineStr"/>
       <c r="AF121" t="inlineStr"/>
       <c r="AG121" t="inlineStr"/>
+      <c r="AH121" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -11851,6 +12239,12 @@
       <c r="AE122" t="inlineStr"/>
       <c r="AF122" t="inlineStr"/>
       <c r="AG122" t="inlineStr"/>
+      <c r="AH122" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -11920,6 +12314,8 @@
       <c r="AE123" t="inlineStr"/>
       <c r="AF123" t="inlineStr"/>
       <c r="AG123" t="inlineStr"/>
+      <c r="AH123" t="inlineStr"/>
+      <c r="AI123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -11989,6 +12385,8 @@
       <c r="AE124" t="inlineStr"/>
       <c r="AF124" t="inlineStr"/>
       <c r="AG124" t="inlineStr"/>
+      <c r="AH124" t="inlineStr"/>
+      <c r="AI124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -12066,6 +12464,8 @@
       <c r="AE125" t="inlineStr"/>
       <c r="AF125" t="inlineStr"/>
       <c r="AG125" t="inlineStr"/>
+      <c r="AH125" t="inlineStr"/>
+      <c r="AI125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -12171,6 +12571,12 @@
       <c r="AE126" t="inlineStr"/>
       <c r="AF126" t="inlineStr"/>
       <c r="AG126" t="inlineStr"/>
+      <c r="AH126" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -12272,6 +12678,12 @@
       <c r="AE127" t="inlineStr"/>
       <c r="AF127" t="inlineStr"/>
       <c r="AG127" t="inlineStr"/>
+      <c r="AH127" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -12365,6 +12777,12 @@
       <c r="AE128" t="inlineStr"/>
       <c r="AF128" t="inlineStr"/>
       <c r="AG128" t="inlineStr"/>
+      <c r="AH128" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -12446,6 +12864,12 @@
       <c r="AE129" t="inlineStr"/>
       <c r="AF129" t="inlineStr"/>
       <c r="AG129" t="inlineStr"/>
+      <c r="AH129" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -12531,6 +12955,12 @@
       <c r="AE130" t="inlineStr"/>
       <c r="AF130" t="inlineStr"/>
       <c r="AG130" t="inlineStr"/>
+      <c r="AH130" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -12652,6 +13082,12 @@
       <c r="AE131" t="inlineStr"/>
       <c r="AF131" t="inlineStr"/>
       <c r="AG131" t="inlineStr"/>
+      <c r="AH131" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -12789,6 +13225,12 @@
       <c r="AE132" t="inlineStr"/>
       <c r="AF132" t="inlineStr"/>
       <c r="AG132" t="inlineStr"/>
+      <c r="AH132" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -12926,6 +13368,12 @@
       <c r="AE133" t="inlineStr"/>
       <c r="AF133" t="inlineStr"/>
       <c r="AG133" t="inlineStr"/>
+      <c r="AH133" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -13059,6 +13507,12 @@
       <c r="AE134" t="inlineStr"/>
       <c r="AF134" t="inlineStr"/>
       <c r="AG134" t="inlineStr"/>
+      <c r="AH134" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -13140,6 +13594,12 @@
       <c r="AE135" t="inlineStr"/>
       <c r="AF135" t="inlineStr"/>
       <c r="AG135" t="inlineStr"/>
+      <c r="AH135" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -13217,6 +13677,12 @@
       <c r="AE136" t="inlineStr"/>
       <c r="AF136" t="inlineStr"/>
       <c r="AG136" t="inlineStr"/>
+      <c r="AH136" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -13306,6 +13772,16 @@
       <c r="AE137" t="inlineStr"/>
       <c r="AF137" t="inlineStr"/>
       <c r="AG137" t="inlineStr"/>
+      <c r="AH137" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI137" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -13391,6 +13867,16 @@
       <c r="AE138" t="inlineStr"/>
       <c r="AF138" t="inlineStr"/>
       <c r="AG138" t="inlineStr"/>
+      <c r="AH138" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI138" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -13476,6 +13962,12 @@
       <c r="AE139" t="inlineStr"/>
       <c r="AF139" t="inlineStr"/>
       <c r="AG139" t="inlineStr"/>
+      <c r="AH139" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -13561,6 +14053,12 @@
       <c r="AE140" t="inlineStr"/>
       <c r="AF140" t="inlineStr"/>
       <c r="AG140" t="inlineStr"/>
+      <c r="AH140" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -13638,6 +14136,8 @@
       <c r="AE141" t="inlineStr"/>
       <c r="AF141" t="inlineStr"/>
       <c r="AG141" t="inlineStr"/>
+      <c r="AH141" t="inlineStr"/>
+      <c r="AI141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -13751,6 +14251,12 @@
       <c r="AE142" t="inlineStr"/>
       <c r="AF142" t="inlineStr"/>
       <c r="AG142" t="inlineStr"/>
+      <c r="AH142" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -13864,6 +14370,12 @@
       <c r="AE143" t="inlineStr"/>
       <c r="AF143" t="inlineStr"/>
       <c r="AG143" t="inlineStr"/>
+      <c r="AH143" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -13981,6 +14493,12 @@
       <c r="AE144" t="inlineStr"/>
       <c r="AF144" t="inlineStr"/>
       <c r="AG144" t="inlineStr"/>
+      <c r="AH144" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -14042,6 +14560,8 @@
       <c r="AE145" t="inlineStr"/>
       <c r="AF145" t="inlineStr"/>
       <c r="AG145" t="inlineStr"/>
+      <c r="AH145" t="inlineStr"/>
+      <c r="AI145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -14111,6 +14631,8 @@
       <c r="AE146" t="inlineStr"/>
       <c r="AF146" t="inlineStr"/>
       <c r="AG146" t="inlineStr"/>
+      <c r="AH146" t="inlineStr"/>
+      <c r="AI146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -14176,6 +14698,8 @@
       <c r="AE147" t="inlineStr"/>
       <c r="AF147" t="inlineStr"/>
       <c r="AG147" t="inlineStr"/>
+      <c r="AH147" t="inlineStr"/>
+      <c r="AI147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -14241,6 +14765,8 @@
       <c r="AE148" t="inlineStr"/>
       <c r="AF148" t="inlineStr"/>
       <c r="AG148" t="inlineStr"/>
+      <c r="AH148" t="inlineStr"/>
+      <c r="AI148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -14310,6 +14836,8 @@
       <c r="AE149" t="inlineStr"/>
       <c r="AF149" t="inlineStr"/>
       <c r="AG149" t="inlineStr"/>
+      <c r="AH149" t="inlineStr"/>
+      <c r="AI149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -14387,6 +14915,8 @@
       <c r="AE150" t="inlineStr"/>
       <c r="AF150" t="inlineStr"/>
       <c r="AG150" t="inlineStr"/>
+      <c r="AH150" t="inlineStr"/>
+      <c r="AI150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -14452,6 +14982,8 @@
       <c r="AE151" t="inlineStr"/>
       <c r="AF151" t="inlineStr"/>
       <c r="AG151" t="inlineStr"/>
+      <c r="AH151" t="inlineStr"/>
+      <c r="AI151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -14537,6 +15069,12 @@
       <c r="AE152" t="inlineStr"/>
       <c r="AF152" t="inlineStr"/>
       <c r="AG152" t="inlineStr"/>
+      <c r="AH152" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -14630,6 +15168,12 @@
       <c r="AE153" t="inlineStr"/>
       <c r="AF153" t="inlineStr"/>
       <c r="AG153" t="inlineStr"/>
+      <c r="AH153" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -14739,6 +15283,12 @@
       <c r="AE154" t="inlineStr"/>
       <c r="AF154" t="inlineStr"/>
       <c r="AG154" t="inlineStr"/>
+      <c r="AH154" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -14844,6 +15394,12 @@
       <c r="AE155" t="inlineStr"/>
       <c r="AF155" t="inlineStr"/>
       <c r="AG155" t="inlineStr"/>
+      <c r="AH155" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -14949,6 +15505,12 @@
       <c r="AE156" t="inlineStr"/>
       <c r="AF156" t="inlineStr"/>
       <c r="AG156" t="inlineStr"/>
+      <c r="AH156" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -15034,6 +15596,16 @@
       <c r="AE157" t="inlineStr"/>
       <c r="AF157" t="inlineStr"/>
       <c r="AG157" t="inlineStr"/>
+      <c r="AH157" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI157" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -15115,6 +15687,12 @@
       <c r="AE158" t="inlineStr"/>
       <c r="AF158" t="inlineStr"/>
       <c r="AG158" t="inlineStr"/>
+      <c r="AH158" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -15196,6 +15774,12 @@
       <c r="AE159" t="inlineStr"/>
       <c r="AF159" t="inlineStr"/>
       <c r="AG159" t="inlineStr"/>
+      <c r="AH159" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -15277,6 +15861,12 @@
       <c r="AE160" t="inlineStr"/>
       <c r="AF160" t="inlineStr"/>
       <c r="AG160" t="inlineStr"/>
+      <c r="AH160" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -15366,6 +15956,12 @@
       <c r="AE161" t="inlineStr"/>
       <c r="AF161" t="inlineStr"/>
       <c r="AG161" t="inlineStr"/>
+      <c r="AH161" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -15443,6 +16039,16 @@
       <c r="AE162" t="inlineStr"/>
       <c r="AF162" t="inlineStr"/>
       <c r="AG162" t="inlineStr"/>
+      <c r="AH162" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI162" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -15520,6 +16126,16 @@
       <c r="AE163" t="inlineStr"/>
       <c r="AF163" t="inlineStr"/>
       <c r="AG163" t="inlineStr"/>
+      <c r="AH163" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI163" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -15593,6 +16209,16 @@
       <c r="AE164" t="inlineStr"/>
       <c r="AF164" t="inlineStr"/>
       <c r="AG164" t="inlineStr"/>
+      <c r="AH164" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI164" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -15670,6 +16296,12 @@
       <c r="AE165" t="inlineStr"/>
       <c r="AF165" t="inlineStr"/>
       <c r="AG165" t="inlineStr"/>
+      <c r="AH165" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -15743,6 +16375,16 @@
       <c r="AE166" t="inlineStr"/>
       <c r="AF166" t="inlineStr"/>
       <c r="AG166" t="inlineStr"/>
+      <c r="AH166" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI166" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -15824,6 +16466,16 @@
       <c r="AE167" t="inlineStr"/>
       <c r="AF167" t="inlineStr"/>
       <c r="AG167" t="inlineStr"/>
+      <c r="AH167" t="inlineStr">
+        <is>
+          <t>iso_001_barrial_060101003003002_Centro_de_embarazas</t>
+        </is>
+      </c>
+      <c r="AI167" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -15901,6 +16553,12 @@
       <c r="AE168" t="inlineStr"/>
       <c r="AF168" t="inlineStr"/>
       <c r="AG168" t="inlineStr"/>
+      <c r="AH168" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -15982,6 +16640,12 @@
       <c r="AE169" t="inlineStr"/>
       <c r="AF169" t="inlineStr"/>
       <c r="AG169" t="inlineStr"/>
+      <c r="AH169" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -16071,6 +16735,12 @@
       <c r="AE170" t="inlineStr"/>
       <c r="AF170" t="inlineStr"/>
       <c r="AG170" t="inlineStr"/>
+      <c r="AH170" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -16168,6 +16838,12 @@
       <c r="AE171" t="inlineStr"/>
       <c r="AF171" t="inlineStr"/>
       <c r="AG171" t="inlineStr"/>
+      <c r="AH171" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -16233,6 +16909,8 @@
       <c r="AE172" t="inlineStr"/>
       <c r="AF172" t="inlineStr"/>
       <c r="AG172" t="inlineStr"/>
+      <c r="AH172" t="inlineStr"/>
+      <c r="AI172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -16294,6 +16972,8 @@
       <c r="AE173" t="inlineStr"/>
       <c r="AF173" t="inlineStr"/>
       <c r="AG173" t="inlineStr"/>
+      <c r="AH173" t="inlineStr"/>
+      <c r="AI173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -16403,6 +17083,12 @@
       <c r="AE174" t="inlineStr"/>
       <c r="AF174" t="inlineStr"/>
       <c r="AG174" t="inlineStr"/>
+      <c r="AH174" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -16516,6 +17202,12 @@
       <c r="AE175" t="inlineStr"/>
       <c r="AF175" t="inlineStr"/>
       <c r="AG175" t="inlineStr"/>
+      <c r="AH175" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -16637,6 +17329,12 @@
       <c r="AE176" t="inlineStr"/>
       <c r="AF176" t="inlineStr"/>
       <c r="AG176" t="inlineStr"/>
+      <c r="AH176" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -16750,6 +17448,12 @@
       <c r="AE177" t="inlineStr"/>
       <c r="AF177" t="inlineStr"/>
       <c r="AG177" t="inlineStr"/>
+      <c r="AH177" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -16855,6 +17559,12 @@
       <c r="AE178" t="inlineStr"/>
       <c r="AF178" t="inlineStr"/>
       <c r="AG178" t="inlineStr"/>
+      <c r="AH178" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -16976,6 +17686,12 @@
       <c r="AE179" t="inlineStr"/>
       <c r="AF179" t="inlineStr"/>
       <c r="AG179" t="inlineStr"/>
+      <c r="AH179" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -17109,6 +17825,12 @@
       <c r="AE180" t="inlineStr"/>
       <c r="AF180" t="inlineStr"/>
       <c r="AG180" t="inlineStr"/>
+      <c r="AH180" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -17242,6 +17964,12 @@
       <c r="AE181" t="inlineStr"/>
       <c r="AF181" t="inlineStr"/>
       <c r="AG181" t="inlineStr"/>
+      <c r="AH181" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -17379,6 +18107,8 @@
       <c r="AE182" t="inlineStr"/>
       <c r="AF182" t="inlineStr"/>
       <c r="AG182" t="inlineStr"/>
+      <c r="AH182" t="inlineStr"/>
+      <c r="AI182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -17496,6 +18226,12 @@
       <c r="AE183" t="inlineStr"/>
       <c r="AF183" t="inlineStr"/>
       <c r="AG183" t="inlineStr"/>
+      <c r="AH183" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -17609,6 +18345,12 @@
       <c r="AE184" t="inlineStr"/>
       <c r="AF184" t="inlineStr"/>
       <c r="AG184" t="inlineStr"/>
+      <c r="AH184" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -17726,6 +18468,12 @@
       <c r="AE185" t="inlineStr"/>
       <c r="AF185" t="inlineStr"/>
       <c r="AG185" t="inlineStr"/>
+      <c r="AH185" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -17851,6 +18599,12 @@
       <c r="AE186" t="inlineStr"/>
       <c r="AF186" t="inlineStr"/>
       <c r="AG186" t="inlineStr"/>
+      <c r="AH186" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -17912,6 +18666,8 @@
       <c r="AE187" t="inlineStr"/>
       <c r="AF187" t="inlineStr"/>
       <c r="AG187" t="inlineStr"/>
+      <c r="AH187" t="inlineStr"/>
+      <c r="AI187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -17973,6 +18729,8 @@
       <c r="AE188" t="inlineStr"/>
       <c r="AF188" t="inlineStr"/>
       <c r="AG188" t="inlineStr"/>
+      <c r="AH188" t="inlineStr"/>
+      <c r="AI188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -18082,6 +18840,12 @@
       <c r="AE189" t="inlineStr"/>
       <c r="AF189" t="inlineStr"/>
       <c r="AG189" t="inlineStr"/>
+      <c r="AH189" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -18203,6 +18967,12 @@
       <c r="AE190" t="inlineStr"/>
       <c r="AF190" t="inlineStr"/>
       <c r="AG190" t="inlineStr"/>
+      <c r="AH190" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -18324,6 +19094,12 @@
       <c r="AE191" t="inlineStr"/>
       <c r="AF191" t="inlineStr"/>
       <c r="AG191" t="inlineStr"/>
+      <c r="AH191" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -18453,6 +19229,8 @@
       <c r="AE192" t="inlineStr"/>
       <c r="AF192" t="inlineStr"/>
       <c r="AG192" t="inlineStr"/>
+      <c r="AH192" t="inlineStr"/>
+      <c r="AI192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -18578,6 +19356,8 @@
       <c r="AE193" t="inlineStr"/>
       <c r="AF193" t="inlineStr"/>
       <c r="AG193" t="inlineStr"/>
+      <c r="AH193" t="inlineStr"/>
+      <c r="AI193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -18691,6 +19471,8 @@
       <c r="AE194" t="inlineStr"/>
       <c r="AF194" t="inlineStr"/>
       <c r="AG194" t="inlineStr"/>
+      <c r="AH194" t="inlineStr"/>
+      <c r="AI194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -18816,6 +19598,12 @@
       <c r="AE195" t="inlineStr"/>
       <c r="AF195" t="inlineStr"/>
       <c r="AG195" t="inlineStr"/>
+      <c r="AH195" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -18933,6 +19721,12 @@
       <c r="AE196" t="inlineStr"/>
       <c r="AF196" t="inlineStr"/>
       <c r="AG196" t="inlineStr"/>
+      <c r="AH196" t="inlineStr">
+        <is>
+          <t>iso_002_zonal_060101003003002_Subcentro_de_Salud_Municipal</t>
+        </is>
+      </c>
+      <c r="AI196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -19002,6 +19796,8 @@
       <c r="AE197" t="inlineStr"/>
       <c r="AF197" t="inlineStr"/>
       <c r="AG197" t="inlineStr"/>
+      <c r="AH197" t="inlineStr"/>
+      <c r="AI197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -19063,9 +19859,11 @@
       <c r="AE198" t="inlineStr"/>
       <c r="AF198" t="inlineStr"/>
       <c r="AG198" t="inlineStr"/>
+      <c r="AH198" t="inlineStr"/>
+      <c r="AI198" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG1"/>
+  <autoFilter ref="A1:AI1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>